<commit_message>
Add motherboard PWM/DC fan headers and fan-header compatibility checks.
Split FanConnectors into PwmFanHeaders and DcFanHeaders, and reject builds when chassis fans exceed available headers after daisy-chain grouping.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Datasheets/PcBuilder-Import-Motherboards.xlsx
+++ b/Datasheets/PcBuilder-Import-Motherboards.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q88"/>
+  <dimension ref="A1:R88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,45 +462,50 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>FanConnectors</t>
+          <t>PwmFanHeaders</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>DcFanHeaders</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>EpsConnectors</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>WidthMm</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>HeightMm</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>DdrGeneration</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>RamFormFactor</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>FormFactor</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>WifiEnabled</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>BluetoothEnabled</t>
         </is>
@@ -543,33 +548,36 @@
         <v>3</v>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" t="n">
         <v>244</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>221</v>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P2" t="b">
-        <v>1</v>
-      </c>
       <c r="Q2" t="b">
+        <v>1</v>
+      </c>
+      <c r="R2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -610,33 +618,36 @@
         <v>3</v>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" t="n">
         <v>244</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>211</v>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P3" t="b">
-        <v>1</v>
-      </c>
       <c r="Q3" t="b">
+        <v>1</v>
+      </c>
+      <c r="R3" t="b">
         <v>1</v>
       </c>
     </row>
@@ -677,33 +688,36 @@
         <v>2</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="n">
         <v>244</v>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>211</v>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Ddr4</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P4" t="b">
-        <v>1</v>
-      </c>
       <c r="Q4" t="b">
+        <v>1</v>
+      </c>
+      <c r="R4" t="b">
         <v>1</v>
       </c>
     </row>
@@ -744,33 +758,36 @@
         <v>4</v>
       </c>
       <c r="J5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="n">
         <v>244</v>
       </c>
-      <c r="L5" t="n">
+      <c r="M5" t="n">
         <v>221</v>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P5" t="b">
-        <v>1</v>
-      </c>
       <c r="Q5" t="b">
+        <v>1</v>
+      </c>
+      <c r="R5" t="b">
         <v>1</v>
       </c>
     </row>
@@ -811,33 +828,36 @@
         <v>3</v>
       </c>
       <c r="J6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="n">
         <v>244</v>
       </c>
-      <c r="L6" t="n">
+      <c r="M6" t="n">
         <v>222</v>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P6" t="b">
-        <v>1</v>
-      </c>
       <c r="Q6" t="b">
+        <v>1</v>
+      </c>
+      <c r="R6" t="b">
         <v>1</v>
       </c>
     </row>
@@ -878,33 +898,36 @@
         <v>2</v>
       </c>
       <c r="J7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" t="n">
         <v>226</v>
       </c>
-      <c r="L7" t="n">
+      <c r="M7" t="n">
         <v>221</v>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Ddr4</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P7" t="b">
-        <v>0</v>
-      </c>
       <c r="Q7" t="b">
+        <v>0</v>
+      </c>
+      <c r="R7" t="b">
         <v>0</v>
       </c>
     </row>
@@ -945,33 +968,36 @@
         <v>2</v>
       </c>
       <c r="J8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
         <v>226</v>
       </c>
-      <c r="L8" t="n">
+      <c r="M8" t="n">
         <v>221</v>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P8" t="b">
-        <v>0</v>
-      </c>
       <c r="Q8" t="b">
+        <v>0</v>
+      </c>
+      <c r="R8" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1012,33 +1038,36 @@
         <v>6</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>244</v>
+        <v>1</v>
       </c>
       <c r="L9" t="n">
         <v>244</v>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M9" t="n">
+        <v>244</v>
+      </c>
+      <c r="N9" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P9" t="b">
-        <v>1</v>
-      </c>
       <c r="Q9" t="b">
+        <v>1</v>
+      </c>
+      <c r="R9" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1079,33 +1108,36 @@
         <v>2</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="n">
         <v>234</v>
       </c>
-      <c r="L10" t="n">
+      <c r="M10" t="n">
         <v>203</v>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>Ddr4</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P10" t="b">
-        <v>0</v>
-      </c>
       <c r="Q10" t="b">
+        <v>0</v>
+      </c>
+      <c r="R10" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1146,33 +1178,36 @@
         <v>3</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
         <v>244</v>
       </c>
-      <c r="L11" t="n">
+      <c r="M11" t="n">
         <v>222</v>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P11" t="b">
-        <v>0</v>
-      </c>
       <c r="Q11" t="b">
+        <v>0</v>
+      </c>
+      <c r="R11" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1213,33 +1248,36 @@
         <v>7</v>
       </c>
       <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
         <v>2</v>
       </c>
-      <c r="K12" t="n">
+      <c r="L12" t="n">
         <v>305</v>
       </c>
-      <c r="L12" t="n">
+      <c r="M12" t="n">
         <v>244</v>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P12" t="b">
-        <v>1</v>
-      </c>
       <c r="Q12" t="b">
+        <v>1</v>
+      </c>
+      <c r="R12" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1280,33 +1318,36 @@
         <v>7</v>
       </c>
       <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
         <v>2</v>
       </c>
-      <c r="K13" t="n">
+      <c r="L13" t="n">
         <v>305</v>
       </c>
-      <c r="L13" t="n">
+      <c r="M13" t="n">
         <v>244</v>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P13" t="b">
-        <v>1</v>
-      </c>
       <c r="Q13" t="b">
+        <v>1</v>
+      </c>
+      <c r="R13" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1347,33 +1388,36 @@
         <v>5</v>
       </c>
       <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
         <v>2</v>
       </c>
-      <c r="K14" t="n">
+      <c r="L14" t="n">
         <v>305</v>
       </c>
-      <c r="L14" t="n">
+      <c r="M14" t="n">
         <v>244</v>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P14" t="b">
-        <v>1</v>
-      </c>
       <c r="Q14" t="b">
+        <v>1</v>
+      </c>
+      <c r="R14" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1414,33 +1458,36 @@
         <v>8</v>
       </c>
       <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
         <v>2</v>
       </c>
-      <c r="K15" t="n">
+      <c r="L15" t="n">
         <v>305</v>
       </c>
-      <c r="L15" t="n">
+      <c r="M15" t="n">
         <v>244</v>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="P15" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P15" t="b">
-        <v>1</v>
-      </c>
       <c r="Q15" t="b">
+        <v>1</v>
+      </c>
+      <c r="R15" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1481,33 +1528,36 @@
         <v>7</v>
       </c>
       <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
         <v>2</v>
       </c>
-      <c r="K16" t="n">
+      <c r="L16" t="n">
         <v>305</v>
       </c>
-      <c r="L16" t="n">
+      <c r="M16" t="n">
         <v>244</v>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P16" t="b">
-        <v>1</v>
-      </c>
       <c r="Q16" t="b">
+        <v>1</v>
+      </c>
+      <c r="R16" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1548,33 +1598,36 @@
         <v>8</v>
       </c>
       <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
         <v>2</v>
       </c>
-      <c r="K17" t="n">
+      <c r="L17" t="n">
         <v>305</v>
       </c>
-      <c r="L17" t="n">
+      <c r="M17" t="n">
         <v>244</v>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="P17" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P17" t="b">
-        <v>1</v>
-      </c>
       <c r="Q17" t="b">
+        <v>1</v>
+      </c>
+      <c r="R17" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1615,33 +1668,36 @@
         <v>8</v>
       </c>
       <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
         <v>2</v>
       </c>
-      <c r="K18" t="n">
+      <c r="L18" t="n">
         <v>305</v>
       </c>
-      <c r="L18" t="n">
+      <c r="M18" t="n">
         <v>244</v>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
+      <c r="P18" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P18" t="b">
-        <v>1</v>
-      </c>
       <c r="Q18" t="b">
+        <v>1</v>
+      </c>
+      <c r="R18" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1682,33 +1738,36 @@
         <v>5</v>
       </c>
       <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
         <v>2</v>
-      </c>
-      <c r="K19" t="n">
-        <v>244</v>
       </c>
       <c r="L19" t="n">
         <v>244</v>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="M19" t="n">
+        <v>244</v>
+      </c>
+      <c r="N19" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="P19" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P19" t="b">
-        <v>1</v>
-      </c>
       <c r="Q19" t="b">
+        <v>1</v>
+      </c>
+      <c r="R19" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1749,33 +1808,36 @@
         <v>6</v>
       </c>
       <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
         <v>2</v>
-      </c>
-      <c r="K20" t="n">
-        <v>244</v>
       </c>
       <c r="L20" t="n">
         <v>244</v>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="M20" t="n">
+        <v>244</v>
+      </c>
+      <c r="N20" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
+      <c r="P20" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P20" t="b">
-        <v>1</v>
-      </c>
       <c r="Q20" t="b">
+        <v>1</v>
+      </c>
+      <c r="R20" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1816,33 +1878,36 @@
         <v>6</v>
       </c>
       <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
         <v>2</v>
-      </c>
-      <c r="K21" t="n">
-        <v>244</v>
       </c>
       <c r="L21" t="n">
         <v>244</v>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="M21" t="n">
+        <v>244</v>
+      </c>
+      <c r="N21" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
+      <c r="P21" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P21" t="b">
-        <v>1</v>
-      </c>
       <c r="Q21" t="b">
+        <v>1</v>
+      </c>
+      <c r="R21" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1883,33 +1948,36 @@
         <v>7</v>
       </c>
       <c r="J22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
         <v>2</v>
       </c>
-      <c r="K22" t="n">
+      <c r="L22" t="n">
         <v>305</v>
       </c>
-      <c r="L22" t="n">
+      <c r="M22" t="n">
         <v>244</v>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="P22" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P22" t="b">
-        <v>1</v>
-      </c>
       <c r="Q22" t="b">
+        <v>1</v>
+      </c>
+      <c r="R22" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1950,33 +2018,36 @@
         <v>7</v>
       </c>
       <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
         <v>2</v>
       </c>
-      <c r="K23" t="n">
+      <c r="L23" t="n">
         <v>305</v>
       </c>
-      <c r="L23" t="n">
+      <c r="M23" t="n">
         <v>244</v>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
+      <c r="P23" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P23" t="b">
-        <v>1</v>
-      </c>
       <c r="Q23" t="b">
+        <v>1</v>
+      </c>
+      <c r="R23" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2017,33 +2088,36 @@
         <v>7</v>
       </c>
       <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
         <v>2</v>
       </c>
-      <c r="K24" t="n">
+      <c r="L24" t="n">
         <v>305</v>
       </c>
-      <c r="L24" t="n">
+      <c r="M24" t="n">
         <v>244</v>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
+      <c r="O24" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr">
+      <c r="P24" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P24" t="b">
-        <v>1</v>
-      </c>
       <c r="Q24" t="b">
+        <v>1</v>
+      </c>
+      <c r="R24" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2084,33 +2158,36 @@
         <v>7</v>
       </c>
       <c r="J25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
         <v>2</v>
       </c>
-      <c r="K25" t="n">
+      <c r="L25" t="n">
         <v>305</v>
       </c>
-      <c r="L25" t="n">
+      <c r="M25" t="n">
         <v>244</v>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
+      <c r="O25" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr">
+      <c r="P25" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P25" t="b">
-        <v>1</v>
-      </c>
       <c r="Q25" t="b">
+        <v>1</v>
+      </c>
+      <c r="R25" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2151,33 +2228,36 @@
         <v>3</v>
       </c>
       <c r="J26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K26" t="n">
+        <v>1</v>
+      </c>
+      <c r="L26" t="n">
         <v>230</v>
       </c>
-      <c r="L26" t="n">
+      <c r="M26" t="n">
         <v>201</v>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>Ddr4</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
+      <c r="O26" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr">
+      <c r="P26" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P26" t="b">
-        <v>0</v>
-      </c>
       <c r="Q26" t="b">
+        <v>0</v>
+      </c>
+      <c r="R26" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2218,33 +2298,36 @@
         <v>4</v>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" t="n">
+        <v>1</v>
+      </c>
+      <c r="L27" t="n">
         <v>244</v>
       </c>
-      <c r="L27" t="n">
+      <c r="M27" t="n">
         <v>226</v>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
+      <c r="O27" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr">
+      <c r="P27" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P27" t="b">
-        <v>1</v>
-      </c>
       <c r="Q27" t="b">
+        <v>1</v>
+      </c>
+      <c r="R27" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2285,33 +2368,36 @@
         <v>4</v>
       </c>
       <c r="J28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K28" t="n">
+        <v>1</v>
+      </c>
+      <c r="L28" t="n">
         <v>244</v>
       </c>
-      <c r="L28" t="n">
+      <c r="M28" t="n">
         <v>201</v>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="N28" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
+      <c r="O28" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr">
+      <c r="P28" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P28" t="b">
-        <v>0</v>
-      </c>
       <c r="Q28" t="b">
+        <v>0</v>
+      </c>
+      <c r="R28" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2352,33 +2438,36 @@
         <v>5</v>
       </c>
       <c r="J29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="n">
         <v>2</v>
-      </c>
-      <c r="K29" t="n">
-        <v>244</v>
       </c>
       <c r="L29" t="n">
         <v>244</v>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="M29" t="n">
+        <v>244</v>
+      </c>
+      <c r="N29" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
+      <c r="O29" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr">
+      <c r="P29" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P29" t="b">
-        <v>0</v>
-      </c>
       <c r="Q29" t="b">
+        <v>0</v>
+      </c>
+      <c r="R29" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2419,33 +2508,36 @@
         <v>4</v>
       </c>
       <c r="J30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K30" t="n">
+        <v>1</v>
+      </c>
+      <c r="L30" t="n">
         <v>244</v>
       </c>
-      <c r="L30" t="n">
+      <c r="M30" t="n">
         <v>226</v>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
+      <c r="O30" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr">
+      <c r="P30" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P30" t="b">
-        <v>1</v>
-      </c>
       <c r="Q30" t="b">
+        <v>1</v>
+      </c>
+      <c r="R30" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2486,33 +2578,36 @@
         <v>7</v>
       </c>
       <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
         <v>2</v>
       </c>
-      <c r="K31" t="n">
+      <c r="L31" t="n">
         <v>305</v>
       </c>
-      <c r="L31" t="n">
+      <c r="M31" t="n">
         <v>244</v>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
+      <c r="O31" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr">
+      <c r="P31" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P31" t="b">
-        <v>1</v>
-      </c>
       <c r="Q31" t="b">
+        <v>1</v>
+      </c>
+      <c r="R31" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2553,33 +2648,36 @@
         <v>5</v>
       </c>
       <c r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="n">
         <v>2</v>
       </c>
-      <c r="K32" t="n">
+      <c r="L32" t="n">
         <v>244</v>
       </c>
-      <c r="L32" t="n">
+      <c r="M32" t="n">
         <v>218</v>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="N32" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
+      <c r="O32" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr">
+      <c r="P32" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P32" t="b">
-        <v>1</v>
-      </c>
       <c r="Q32" t="b">
+        <v>1</v>
+      </c>
+      <c r="R32" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2620,33 +2718,36 @@
         <v>7</v>
       </c>
       <c r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="n">
         <v>2</v>
       </c>
-      <c r="K33" t="n">
+      <c r="L33" t="n">
         <v>305</v>
       </c>
-      <c r="L33" t="n">
+      <c r="M33" t="n">
         <v>244</v>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="N33" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
+      <c r="O33" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr">
+      <c r="P33" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P33" t="b">
-        <v>1</v>
-      </c>
       <c r="Q33" t="b">
+        <v>1</v>
+      </c>
+      <c r="R33" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2687,33 +2788,36 @@
         <v>2</v>
       </c>
       <c r="J34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K34" t="n">
+        <v>1</v>
+      </c>
+      <c r="L34" t="n">
         <v>220</v>
       </c>
-      <c r="L34" t="n">
+      <c r="M34" t="n">
         <v>193</v>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="N34" t="inlineStr">
         <is>
           <t>Ddr4</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
+      <c r="O34" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr">
+      <c r="P34" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P34" t="b">
-        <v>0</v>
-      </c>
       <c r="Q34" t="b">
+        <v>0</v>
+      </c>
+      <c r="R34" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2754,33 +2858,36 @@
         <v>2</v>
       </c>
       <c r="J35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K35" t="n">
+        <v>1</v>
+      </c>
+      <c r="L35" t="n">
         <v>244</v>
       </c>
-      <c r="L35" t="n">
+      <c r="M35" t="n">
         <v>193</v>
       </c>
-      <c r="M35" t="inlineStr">
+      <c r="N35" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr">
+      <c r="O35" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr">
+      <c r="P35" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P35" t="b">
-        <v>1</v>
-      </c>
       <c r="Q35" t="b">
+        <v>1</v>
+      </c>
+      <c r="R35" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2821,33 +2928,36 @@
         <v>5</v>
       </c>
       <c r="J36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K36" t="n">
+        <v>1</v>
+      </c>
+      <c r="L36" t="n">
         <v>305</v>
       </c>
-      <c r="L36" t="n">
+      <c r="M36" t="n">
         <v>229</v>
       </c>
-      <c r="M36" t="inlineStr">
+      <c r="N36" t="inlineStr">
         <is>
           <t>Ddr4</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr">
+      <c r="O36" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr">
+      <c r="P36" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P36" t="b">
-        <v>0</v>
-      </c>
       <c r="Q36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R36" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2888,33 +2998,36 @@
         <v>6</v>
       </c>
       <c r="J37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" t="n">
         <v>2</v>
       </c>
-      <c r="K37" t="n">
+      <c r="L37" t="n">
         <v>305</v>
       </c>
-      <c r="L37" t="n">
+      <c r="M37" t="n">
         <v>244</v>
       </c>
-      <c r="M37" t="inlineStr">
+      <c r="N37" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr">
+      <c r="O37" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr">
+      <c r="P37" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P37" t="b">
-        <v>1</v>
-      </c>
       <c r="Q37" t="b">
+        <v>1</v>
+      </c>
+      <c r="R37" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2955,33 +3068,36 @@
         <v>7</v>
       </c>
       <c r="J38" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" t="n">
         <v>2</v>
       </c>
-      <c r="K38" t="n">
+      <c r="L38" t="n">
         <v>305</v>
       </c>
-      <c r="L38" t="n">
+      <c r="M38" t="n">
         <v>244</v>
       </c>
-      <c r="M38" t="inlineStr">
+      <c r="N38" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr">
+      <c r="O38" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr">
+      <c r="P38" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P38" t="b">
-        <v>1</v>
-      </c>
       <c r="Q38" t="b">
+        <v>1</v>
+      </c>
+      <c r="R38" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3022,33 +3138,36 @@
         <v>8</v>
       </c>
       <c r="J39" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" t="n">
         <v>2</v>
       </c>
-      <c r="K39" t="n">
+      <c r="L39" t="n">
         <v>305</v>
       </c>
-      <c r="L39" t="n">
+      <c r="M39" t="n">
         <v>267</v>
       </c>
-      <c r="M39" t="inlineStr">
+      <c r="N39" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr">
+      <c r="O39" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr">
+      <c r="P39" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P39" t="b">
-        <v>1</v>
-      </c>
       <c r="Q39" t="b">
+        <v>1</v>
+      </c>
+      <c r="R39" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3089,33 +3208,36 @@
         <v>7</v>
       </c>
       <c r="J40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" t="n">
         <v>2</v>
       </c>
-      <c r="K40" t="n">
+      <c r="L40" t="n">
         <v>305</v>
       </c>
-      <c r="L40" t="n">
+      <c r="M40" t="n">
         <v>244</v>
       </c>
-      <c r="M40" t="inlineStr">
+      <c r="N40" t="inlineStr">
         <is>
           <t>Ddr4</t>
         </is>
       </c>
-      <c r="N40" t="inlineStr">
+      <c r="O40" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O40" t="inlineStr">
+      <c r="P40" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P40" t="b">
-        <v>0</v>
-      </c>
       <c r="Q40" t="b">
+        <v>0</v>
+      </c>
+      <c r="R40" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3156,33 +3278,36 @@
         <v>3</v>
       </c>
       <c r="J41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K41" t="n">
-        <v>170</v>
+        <v>1</v>
       </c>
       <c r="L41" t="n">
         <v>170</v>
       </c>
-      <c r="M41" t="inlineStr">
+      <c r="M41" t="n">
+        <v>170</v>
+      </c>
+      <c r="N41" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr">
+      <c r="O41" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr">
+      <c r="P41" t="inlineStr">
         <is>
           <t>Mitx</t>
         </is>
       </c>
-      <c r="P41" t="b">
-        <v>1</v>
-      </c>
       <c r="Q41" t="b">
+        <v>1</v>
+      </c>
+      <c r="R41" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3223,33 +3348,36 @@
         <v>8</v>
       </c>
       <c r="J42" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" t="n">
         <v>2</v>
       </c>
-      <c r="K42" t="n">
+      <c r="L42" t="n">
         <v>305</v>
       </c>
-      <c r="L42" t="n">
+      <c r="M42" t="n">
         <v>244</v>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="N42" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr">
+      <c r="O42" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr">
+      <c r="P42" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P42" t="b">
-        <v>1</v>
-      </c>
       <c r="Q42" t="b">
+        <v>1</v>
+      </c>
+      <c r="R42" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3290,33 +3418,36 @@
         <v>8</v>
       </c>
       <c r="J43" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" t="n">
         <v>2</v>
       </c>
-      <c r="K43" t="n">
+      <c r="L43" t="n">
         <v>305</v>
       </c>
-      <c r="L43" t="n">
+      <c r="M43" t="n">
         <v>244</v>
       </c>
-      <c r="M43" t="inlineStr">
+      <c r="N43" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr">
+      <c r="O43" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr">
+      <c r="P43" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P43" t="b">
-        <v>1</v>
-      </c>
       <c r="Q43" t="b">
+        <v>1</v>
+      </c>
+      <c r="R43" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3357,33 +3488,36 @@
         <v>2</v>
       </c>
       <c r="J44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>244</v>
+        <v>1</v>
       </c>
       <c r="L44" t="n">
         <v>244</v>
       </c>
-      <c r="M44" t="inlineStr">
+      <c r="M44" t="n">
+        <v>244</v>
+      </c>
+      <c r="N44" t="inlineStr">
         <is>
           <t>Ddr4</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr">
+      <c r="O44" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr">
+      <c r="P44" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P44" t="b">
-        <v>1</v>
-      </c>
       <c r="Q44" t="b">
+        <v>1</v>
+      </c>
+      <c r="R44" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3424,33 +3558,36 @@
         <v>3</v>
       </c>
       <c r="J45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K45" t="n">
+        <v>1</v>
+      </c>
+      <c r="L45" t="n">
         <v>230</v>
       </c>
-      <c r="L45" t="n">
+      <c r="M45" t="n">
         <v>215</v>
       </c>
-      <c r="M45" t="inlineStr">
+      <c r="N45" t="inlineStr">
         <is>
           <t>Ddr4</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr">
+      <c r="O45" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr">
+      <c r="P45" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P45" t="b">
-        <v>0</v>
-      </c>
       <c r="Q45" t="b">
+        <v>0</v>
+      </c>
+      <c r="R45" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3491,33 +3628,36 @@
         <v>4</v>
       </c>
       <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="n">
         <v>2</v>
-      </c>
-      <c r="K46" t="n">
-        <v>244</v>
       </c>
       <c r="L46" t="n">
         <v>244</v>
       </c>
-      <c r="M46" t="inlineStr">
+      <c r="M46" t="n">
+        <v>244</v>
+      </c>
+      <c r="N46" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr">
+      <c r="O46" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O46" t="inlineStr">
+      <c r="P46" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P46" t="b">
-        <v>1</v>
-      </c>
       <c r="Q46" t="b">
+        <v>1</v>
+      </c>
+      <c r="R46" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3558,33 +3698,36 @@
         <v>4</v>
       </c>
       <c r="J47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K47" t="n">
-        <v>244</v>
+        <v>1</v>
       </c>
       <c r="L47" t="n">
         <v>244</v>
       </c>
-      <c r="M47" t="inlineStr">
+      <c r="M47" t="n">
+        <v>244</v>
+      </c>
+      <c r="N47" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N47" t="inlineStr">
+      <c r="O47" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr">
+      <c r="P47" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P47" t="b">
-        <v>1</v>
-      </c>
       <c r="Q47" t="b">
+        <v>1</v>
+      </c>
+      <c r="R47" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3625,33 +3768,36 @@
         <v>6</v>
       </c>
       <c r="J48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" t="n">
         <v>2</v>
       </c>
-      <c r="K48" t="n">
+      <c r="L48" t="n">
         <v>305</v>
       </c>
-      <c r="L48" t="n">
+      <c r="M48" t="n">
         <v>244</v>
       </c>
-      <c r="M48" t="inlineStr">
+      <c r="N48" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N48" t="inlineStr">
+      <c r="O48" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O48" t="inlineStr">
+      <c r="P48" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P48" t="b">
-        <v>1</v>
-      </c>
       <c r="Q48" t="b">
+        <v>1</v>
+      </c>
+      <c r="R48" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3692,33 +3838,36 @@
         <v>8</v>
       </c>
       <c r="J49" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" t="n">
         <v>2</v>
       </c>
-      <c r="K49" t="n">
+      <c r="L49" t="n">
         <v>305</v>
       </c>
-      <c r="L49" t="n">
+      <c r="M49" t="n">
         <v>244</v>
       </c>
-      <c r="M49" t="inlineStr">
+      <c r="N49" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr">
+      <c r="O49" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O49" t="inlineStr">
+      <c r="P49" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P49" t="b">
-        <v>1</v>
-      </c>
       <c r="Q49" t="b">
+        <v>1</v>
+      </c>
+      <c r="R49" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3759,33 +3908,36 @@
         <v>6</v>
       </c>
       <c r="J50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K50" t="n">
+        <v>1</v>
+      </c>
+      <c r="L50" t="n">
         <v>305</v>
       </c>
-      <c r="L50" t="n">
+      <c r="M50" t="n">
         <v>244</v>
       </c>
-      <c r="M50" t="inlineStr">
+      <c r="N50" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr">
+      <c r="O50" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O50" t="inlineStr">
+      <c r="P50" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P50" t="b">
-        <v>1</v>
-      </c>
       <c r="Q50" t="b">
+        <v>1</v>
+      </c>
+      <c r="R50" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3826,33 +3978,36 @@
         <v>4</v>
       </c>
       <c r="J51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K51" t="n">
+        <v>1</v>
+      </c>
+      <c r="L51" t="n">
         <v>244</v>
       </c>
-      <c r="L51" t="n">
+      <c r="M51" t="n">
         <v>225</v>
       </c>
-      <c r="M51" t="inlineStr">
+      <c r="N51" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N51" t="inlineStr">
+      <c r="O51" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O51" t="inlineStr">
+      <c r="P51" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P51" t="b">
-        <v>1</v>
-      </c>
       <c r="Q51" t="b">
+        <v>1</v>
+      </c>
+      <c r="R51" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3893,33 +4048,36 @@
         <v>3</v>
       </c>
       <c r="J52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K52" t="n">
-        <v>170</v>
+        <v>1</v>
       </c>
       <c r="L52" t="n">
         <v>170</v>
       </c>
-      <c r="M52" t="inlineStr">
+      <c r="M52" t="n">
+        <v>170</v>
+      </c>
+      <c r="N52" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr">
+      <c r="O52" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O52" t="inlineStr">
+      <c r="P52" t="inlineStr">
         <is>
           <t>Mitx</t>
         </is>
       </c>
-      <c r="P52" t="b">
-        <v>1</v>
-      </c>
       <c r="Q52" t="b">
+        <v>1</v>
+      </c>
+      <c r="R52" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3960,33 +4118,36 @@
         <v>3</v>
       </c>
       <c r="J53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K53" t="n">
+        <v>1</v>
+      </c>
+      <c r="L53" t="n">
         <v>223</v>
       </c>
-      <c r="L53" t="n">
+      <c r="M53" t="n">
         <v>193</v>
       </c>
-      <c r="M53" t="inlineStr">
+      <c r="N53" t="inlineStr">
         <is>
           <t>Ddr4</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr">
+      <c r="O53" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O53" t="inlineStr">
+      <c r="P53" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P53" t="b">
-        <v>0</v>
-      </c>
       <c r="Q53" t="b">
+        <v>0</v>
+      </c>
+      <c r="R53" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4027,33 +4188,36 @@
         <v>3</v>
       </c>
       <c r="J54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K54" t="n">
+        <v>1</v>
+      </c>
+      <c r="L54" t="n">
         <v>244</v>
       </c>
-      <c r="L54" t="n">
+      <c r="M54" t="n">
         <v>215</v>
       </c>
-      <c r="M54" t="inlineStr">
+      <c r="N54" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N54" t="inlineStr">
+      <c r="O54" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O54" t="inlineStr">
+      <c r="P54" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P54" t="b">
-        <v>0</v>
-      </c>
       <c r="Q54" t="b">
+        <v>0</v>
+      </c>
+      <c r="R54" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4094,33 +4258,36 @@
         <v>6</v>
       </c>
       <c r="J55" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" t="n">
         <v>2</v>
       </c>
-      <c r="K55" t="n">
+      <c r="L55" t="n">
         <v>305</v>
       </c>
-      <c r="L55" t="n">
+      <c r="M55" t="n">
         <v>244</v>
       </c>
-      <c r="M55" t="inlineStr">
+      <c r="N55" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N55" t="inlineStr">
+      <c r="O55" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O55" t="inlineStr">
+      <c r="P55" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P55" t="b">
-        <v>1</v>
-      </c>
       <c r="Q55" t="b">
+        <v>1</v>
+      </c>
+      <c r="R55" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4161,33 +4328,36 @@
         <v>8</v>
       </c>
       <c r="J56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" t="n">
         <v>2</v>
       </c>
-      <c r="K56" t="n">
+      <c r="L56" t="n">
         <v>305</v>
       </c>
-      <c r="L56" t="n">
+      <c r="M56" t="n">
         <v>244</v>
       </c>
-      <c r="M56" t="inlineStr">
+      <c r="N56" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr">
+      <c r="O56" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O56" t="inlineStr">
+      <c r="P56" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P56" t="b">
-        <v>1</v>
-      </c>
       <c r="Q56" t="b">
+        <v>1</v>
+      </c>
+      <c r="R56" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4228,33 +4398,36 @@
         <v>8</v>
       </c>
       <c r="J57" t="n">
+        <v>0</v>
+      </c>
+      <c r="K57" t="n">
         <v>2</v>
       </c>
-      <c r="K57" t="n">
+      <c r="L57" t="n">
         <v>305</v>
       </c>
-      <c r="L57" t="n">
+      <c r="M57" t="n">
         <v>244</v>
       </c>
-      <c r="M57" t="inlineStr">
+      <c r="N57" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr">
+      <c r="O57" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O57" t="inlineStr">
+      <c r="P57" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P57" t="b">
-        <v>1</v>
-      </c>
       <c r="Q57" t="b">
+        <v>1</v>
+      </c>
+      <c r="R57" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4295,33 +4468,36 @@
         <v>10</v>
       </c>
       <c r="J58" t="n">
+        <v>0</v>
+      </c>
+      <c r="K58" t="n">
         <v>2</v>
       </c>
-      <c r="K58" t="n">
+      <c r="L58" t="n">
         <v>305</v>
       </c>
-      <c r="L58" t="n">
+      <c r="M58" t="n">
         <v>269</v>
       </c>
-      <c r="M58" t="inlineStr">
+      <c r="N58" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N58" t="inlineStr">
+      <c r="O58" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O58" t="inlineStr">
+      <c r="P58" t="inlineStr">
         <is>
           <t>Eatx</t>
         </is>
       </c>
-      <c r="P58" t="b">
-        <v>1</v>
-      </c>
       <c r="Q58" t="b">
+        <v>1</v>
+      </c>
+      <c r="R58" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4362,33 +4538,36 @@
         <v>6</v>
       </c>
       <c r="J59" t="n">
+        <v>0</v>
+      </c>
+      <c r="K59" t="n">
         <v>2</v>
       </c>
-      <c r="K59" t="n">
+      <c r="L59" t="n">
         <v>305</v>
       </c>
-      <c r="L59" t="n">
+      <c r="M59" t="n">
         <v>244</v>
       </c>
-      <c r="M59" t="inlineStr">
+      <c r="N59" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N59" t="inlineStr">
+      <c r="O59" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O59" t="inlineStr">
+      <c r="P59" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P59" t="b">
-        <v>0</v>
-      </c>
       <c r="Q59" t="b">
+        <v>0</v>
+      </c>
+      <c r="R59" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4429,33 +4608,36 @@
         <v>6</v>
       </c>
       <c r="J60" t="n">
+        <v>0</v>
+      </c>
+      <c r="K60" t="n">
         <v>2</v>
       </c>
-      <c r="K60" t="n">
+      <c r="L60" t="n">
         <v>305</v>
       </c>
-      <c r="L60" t="n">
+      <c r="M60" t="n">
         <v>244</v>
       </c>
-      <c r="M60" t="inlineStr">
+      <c r="N60" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N60" t="inlineStr">
+      <c r="O60" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O60" t="inlineStr">
+      <c r="P60" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P60" t="b">
-        <v>1</v>
-      </c>
       <c r="Q60" t="b">
+        <v>1</v>
+      </c>
+      <c r="R60" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4496,33 +4678,36 @@
         <v>10</v>
       </c>
       <c r="J61" t="n">
+        <v>0</v>
+      </c>
+      <c r="K61" t="n">
         <v>2</v>
       </c>
-      <c r="K61" t="n">
+      <c r="L61" t="n">
         <v>305</v>
       </c>
-      <c r="L61" t="n">
+      <c r="M61" t="n">
         <v>244</v>
       </c>
-      <c r="M61" t="inlineStr">
+      <c r="N61" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N61" t="inlineStr">
+      <c r="O61" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O61" t="inlineStr">
+      <c r="P61" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P61" t="b">
-        <v>1</v>
-      </c>
       <c r="Q61" t="b">
+        <v>1</v>
+      </c>
+      <c r="R61" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4563,33 +4748,36 @@
         <v>2</v>
       </c>
       <c r="J62" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K62" t="n">
+        <v>1</v>
+      </c>
+      <c r="L62" t="n">
         <v>243.84</v>
       </c>
-      <c r="L62" t="n">
+      <c r="M62" t="n">
         <v>210</v>
       </c>
-      <c r="M62" t="inlineStr">
+      <c r="N62" t="inlineStr">
         <is>
           <t>Ddr4</t>
         </is>
       </c>
-      <c r="N62" t="inlineStr">
+      <c r="O62" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O62" t="inlineStr">
+      <c r="P62" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P62" t="b">
-        <v>1</v>
-      </c>
       <c r="Q62" t="b">
+        <v>1</v>
+      </c>
+      <c r="R62" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4630,33 +4818,36 @@
         <v>3</v>
       </c>
       <c r="J63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K63" t="n">
+        <v>1</v>
+      </c>
+      <c r="L63" t="n">
         <v>243.84</v>
       </c>
-      <c r="L63" t="n">
+      <c r="M63" t="n">
         <v>211</v>
       </c>
-      <c r="M63" t="inlineStr">
+      <c r="N63" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N63" t="inlineStr">
+      <c r="O63" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O63" t="inlineStr">
+      <c r="P63" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P63" t="b">
-        <v>0</v>
-      </c>
       <c r="Q63" t="b">
+        <v>0</v>
+      </c>
+      <c r="R63" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4697,33 +4888,36 @@
         <v>2</v>
       </c>
       <c r="J64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K64" t="n">
+        <v>1</v>
+      </c>
+      <c r="L64" t="n">
         <v>243.84</v>
       </c>
-      <c r="L64" t="n">
+      <c r="M64" t="n">
         <v>210</v>
       </c>
-      <c r="M64" t="inlineStr">
+      <c r="N64" t="inlineStr">
         <is>
           <t>Ddr4</t>
         </is>
       </c>
-      <c r="N64" t="inlineStr">
+      <c r="O64" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O64" t="inlineStr">
+      <c r="P64" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P64" t="b">
-        <v>1</v>
-      </c>
       <c r="Q64" t="b">
+        <v>1</v>
+      </c>
+      <c r="R64" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4764,33 +4958,36 @@
         <v>4</v>
       </c>
       <c r="J65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K65" t="n">
+        <v>1</v>
+      </c>
+      <c r="L65" t="n">
         <v>243.84</v>
       </c>
-      <c r="L65" t="n">
+      <c r="M65" t="n">
         <v>226</v>
       </c>
-      <c r="M65" t="inlineStr">
+      <c r="N65" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N65" t="inlineStr">
+      <c r="O65" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O65" t="inlineStr">
+      <c r="P65" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P65" t="b">
-        <v>1</v>
-      </c>
       <c r="Q65" t="b">
+        <v>1</v>
+      </c>
+      <c r="R65" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4831,33 +5028,36 @@
         <v>4</v>
       </c>
       <c r="J66" t="n">
+        <v>0</v>
+      </c>
+      <c r="K66" t="n">
         <v>2</v>
-      </c>
-      <c r="K66" t="n">
-        <v>243.84</v>
       </c>
       <c r="L66" t="n">
         <v>243.84</v>
       </c>
-      <c r="M66" t="inlineStr">
+      <c r="M66" t="n">
+        <v>243.84</v>
+      </c>
+      <c r="N66" t="inlineStr">
         <is>
           <t>Ddr4</t>
         </is>
       </c>
-      <c r="N66" t="inlineStr">
+      <c r="O66" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O66" t="inlineStr">
+      <c r="P66" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P66" t="b">
-        <v>1</v>
-      </c>
       <c r="Q66" t="b">
+        <v>1</v>
+      </c>
+      <c r="R66" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4898,33 +5098,36 @@
         <v>4</v>
       </c>
       <c r="J67" t="n">
+        <v>0</v>
+      </c>
+      <c r="K67" t="n">
         <v>2</v>
-      </c>
-      <c r="K67" t="n">
-        <v>243.84</v>
       </c>
       <c r="L67" t="n">
         <v>243.84</v>
       </c>
-      <c r="M67" t="inlineStr">
+      <c r="M67" t="n">
+        <v>243.84</v>
+      </c>
+      <c r="N67" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N67" t="inlineStr">
+      <c r="O67" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O67" t="inlineStr">
+      <c r="P67" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P67" t="b">
-        <v>1</v>
-      </c>
       <c r="Q67" t="b">
+        <v>1</v>
+      </c>
+      <c r="R67" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4965,33 +5168,36 @@
         <v>3</v>
       </c>
       <c r="J68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K68" t="n">
+        <v>1</v>
+      </c>
+      <c r="L68" t="n">
         <v>243.84</v>
       </c>
-      <c r="L68" t="n">
+      <c r="M68" t="n">
         <v>220</v>
       </c>
-      <c r="M68" t="inlineStr">
+      <c r="N68" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N68" t="inlineStr">
+      <c r="O68" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O68" t="inlineStr">
+      <c r="P68" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P68" t="b">
-        <v>1</v>
-      </c>
       <c r="Q68" t="b">
+        <v>1</v>
+      </c>
+      <c r="R68" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5032,33 +5238,36 @@
         <v>6</v>
       </c>
       <c r="J69" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" t="n">
         <v>2</v>
       </c>
-      <c r="K69" t="n">
+      <c r="L69" t="n">
         <v>304.8</v>
       </c>
-      <c r="L69" t="n">
+      <c r="M69" t="n">
         <v>243.84</v>
       </c>
-      <c r="M69" t="inlineStr">
+      <c r="N69" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N69" t="inlineStr">
+      <c r="O69" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O69" t="inlineStr">
+      <c r="P69" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P69" t="b">
-        <v>1</v>
-      </c>
       <c r="Q69" t="b">
+        <v>1</v>
+      </c>
+      <c r="R69" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5099,33 +5308,36 @@
         <v>6</v>
       </c>
       <c r="J70" t="n">
+        <v>0</v>
+      </c>
+      <c r="K70" t="n">
         <v>2</v>
-      </c>
-      <c r="K70" t="n">
-        <v>243.84</v>
       </c>
       <c r="L70" t="n">
         <v>243.84</v>
       </c>
-      <c r="M70" t="inlineStr">
+      <c r="M70" t="n">
+        <v>243.84</v>
+      </c>
+      <c r="N70" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N70" t="inlineStr">
+      <c r="O70" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O70" t="inlineStr">
+      <c r="P70" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P70" t="b">
-        <v>1</v>
-      </c>
       <c r="Q70" t="b">
+        <v>1</v>
+      </c>
+      <c r="R70" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5166,33 +5378,36 @@
         <v>8</v>
       </c>
       <c r="J71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K71" t="n">
         <v>2</v>
       </c>
-      <c r="K71" t="n">
+      <c r="L71" t="n">
         <v>304.8</v>
       </c>
-      <c r="L71" t="n">
+      <c r="M71" t="n">
         <v>243.84</v>
       </c>
-      <c r="M71" t="inlineStr">
+      <c r="N71" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N71" t="inlineStr">
+      <c r="O71" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O71" t="inlineStr">
+      <c r="P71" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P71" t="b">
-        <v>1</v>
-      </c>
       <c r="Q71" t="b">
+        <v>1</v>
+      </c>
+      <c r="R71" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5233,33 +5448,36 @@
         <v>6</v>
       </c>
       <c r="J72" t="n">
+        <v>0</v>
+      </c>
+      <c r="K72" t="n">
         <v>2</v>
       </c>
-      <c r="K72" t="n">
+      <c r="L72" t="n">
         <v>304.8</v>
       </c>
-      <c r="L72" t="n">
+      <c r="M72" t="n">
         <v>243.84</v>
       </c>
-      <c r="M72" t="inlineStr">
+      <c r="N72" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N72" t="inlineStr">
+      <c r="O72" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O72" t="inlineStr">
+      <c r="P72" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P72" t="b">
-        <v>1</v>
-      </c>
       <c r="Q72" t="b">
+        <v>1</v>
+      </c>
+      <c r="R72" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5300,33 +5518,36 @@
         <v>6</v>
       </c>
       <c r="J73" t="n">
+        <v>0</v>
+      </c>
+      <c r="K73" t="n">
         <v>2</v>
-      </c>
-      <c r="K73" t="n">
-        <v>243.84</v>
       </c>
       <c r="L73" t="n">
         <v>243.84</v>
       </c>
-      <c r="M73" t="inlineStr">
+      <c r="M73" t="n">
+        <v>243.84</v>
+      </c>
+      <c r="N73" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N73" t="inlineStr">
+      <c r="O73" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O73" t="inlineStr">
+      <c r="P73" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P73" t="b">
-        <v>1</v>
-      </c>
       <c r="Q73" t="b">
+        <v>1</v>
+      </c>
+      <c r="R73" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5367,33 +5588,36 @@
         <v>3</v>
       </c>
       <c r="J74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K74" t="n">
-        <v>170</v>
+        <v>1</v>
       </c>
       <c r="L74" t="n">
         <v>170</v>
       </c>
-      <c r="M74" t="inlineStr">
+      <c r="M74" t="n">
+        <v>170</v>
+      </c>
+      <c r="N74" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N74" t="inlineStr">
+      <c r="O74" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O74" t="inlineStr">
+      <c r="P74" t="inlineStr">
         <is>
           <t>Mitx</t>
         </is>
       </c>
-      <c r="P74" t="b">
-        <v>1</v>
-      </c>
       <c r="Q74" t="b">
+        <v>1</v>
+      </c>
+      <c r="R74" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5434,33 +5658,36 @@
         <v>2</v>
       </c>
       <c r="J75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K75" t="n">
+        <v>1</v>
+      </c>
+      <c r="L75" t="n">
         <v>236.16</v>
       </c>
-      <c r="L75" t="n">
+      <c r="M75" t="n">
         <v>200</v>
       </c>
-      <c r="M75" t="inlineStr">
+      <c r="N75" t="inlineStr">
         <is>
           <t>Ddr4</t>
         </is>
       </c>
-      <c r="N75" t="inlineStr">
+      <c r="O75" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O75" t="inlineStr">
+      <c r="P75" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P75" t="b">
-        <v>1</v>
-      </c>
       <c r="Q75" t="b">
+        <v>1</v>
+      </c>
+      <c r="R75" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5501,33 +5728,36 @@
         <v>3</v>
       </c>
       <c r="J76" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K76" t="n">
+        <v>1</v>
+      </c>
+      <c r="L76" t="n">
         <v>236.16</v>
       </c>
-      <c r="L76" t="n">
+      <c r="M76" t="n">
         <v>200</v>
       </c>
-      <c r="M76" t="inlineStr">
+      <c r="N76" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N76" t="inlineStr">
+      <c r="O76" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O76" t="inlineStr">
+      <c r="P76" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P76" t="b">
-        <v>0</v>
-      </c>
       <c r="Q76" t="b">
+        <v>0</v>
+      </c>
+      <c r="R76" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5568,33 +5798,36 @@
         <v>3</v>
       </c>
       <c r="J77" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K77" t="n">
+        <v>1</v>
+      </c>
+      <c r="L77" t="n">
         <v>243.84</v>
       </c>
-      <c r="L77" t="n">
+      <c r="M77" t="n">
         <v>220</v>
       </c>
-      <c r="M77" t="inlineStr">
+      <c r="N77" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N77" t="inlineStr">
+      <c r="O77" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O77" t="inlineStr">
+      <c r="P77" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P77" t="b">
-        <v>1</v>
-      </c>
       <c r="Q77" t="b">
+        <v>1</v>
+      </c>
+      <c r="R77" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5635,33 +5868,36 @@
         <v>7</v>
       </c>
       <c r="J78" t="n">
+        <v>0</v>
+      </c>
+      <c r="K78" t="n">
         <v>2</v>
       </c>
-      <c r="K78" t="n">
+      <c r="L78" t="n">
         <v>304.8</v>
       </c>
-      <c r="L78" t="n">
+      <c r="M78" t="n">
         <v>243.84</v>
       </c>
-      <c r="M78" t="inlineStr">
+      <c r="N78" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N78" t="inlineStr">
+      <c r="O78" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O78" t="inlineStr">
+      <c r="P78" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P78" t="b">
-        <v>1</v>
-      </c>
       <c r="Q78" t="b">
+        <v>1</v>
+      </c>
+      <c r="R78" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5702,33 +5938,36 @@
         <v>8</v>
       </c>
       <c r="J79" t="n">
+        <v>0</v>
+      </c>
+      <c r="K79" t="n">
         <v>2</v>
       </c>
-      <c r="K79" t="n">
+      <c r="L79" t="n">
         <v>304.8</v>
       </c>
-      <c r="L79" t="n">
+      <c r="M79" t="n">
         <v>243.84</v>
       </c>
-      <c r="M79" t="inlineStr">
+      <c r="N79" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N79" t="inlineStr">
+      <c r="O79" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O79" t="inlineStr">
+      <c r="P79" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P79" t="b">
-        <v>1</v>
-      </c>
       <c r="Q79" t="b">
+        <v>1</v>
+      </c>
+      <c r="R79" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5769,33 +6008,36 @@
         <v>3</v>
       </c>
       <c r="J80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K80" t="n">
-        <v>170</v>
+        <v>1</v>
       </c>
       <c r="L80" t="n">
         <v>170</v>
       </c>
-      <c r="M80" t="inlineStr">
+      <c r="M80" t="n">
+        <v>170</v>
+      </c>
+      <c r="N80" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N80" t="inlineStr">
+      <c r="O80" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O80" t="inlineStr">
+      <c r="P80" t="inlineStr">
         <is>
           <t>Mitx</t>
         </is>
       </c>
-      <c r="P80" t="b">
-        <v>1</v>
-      </c>
       <c r="Q80" t="b">
+        <v>1</v>
+      </c>
+      <c r="R80" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5836,33 +6078,36 @@
         <v>8</v>
       </c>
       <c r="J81" t="n">
+        <v>0</v>
+      </c>
+      <c r="K81" t="n">
         <v>2</v>
       </c>
-      <c r="K81" t="n">
+      <c r="L81" t="n">
         <v>304.8</v>
       </c>
-      <c r="L81" t="n">
+      <c r="M81" t="n">
         <v>243.84</v>
       </c>
-      <c r="M81" t="inlineStr">
+      <c r="N81" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N81" t="inlineStr">
+      <c r="O81" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O81" t="inlineStr">
+      <c r="P81" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P81" t="b">
-        <v>1</v>
-      </c>
       <c r="Q81" t="b">
+        <v>1</v>
+      </c>
+      <c r="R81" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5903,33 +6148,36 @@
         <v>8</v>
       </c>
       <c r="J82" t="n">
+        <v>0</v>
+      </c>
+      <c r="K82" t="n">
         <v>2</v>
       </c>
-      <c r="K82" t="n">
+      <c r="L82" t="n">
         <v>304.8</v>
       </c>
-      <c r="L82" t="n">
+      <c r="M82" t="n">
         <v>243.84</v>
       </c>
-      <c r="M82" t="inlineStr">
+      <c r="N82" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N82" t="inlineStr">
+      <c r="O82" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O82" t="inlineStr">
+      <c r="P82" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P82" t="b">
-        <v>1</v>
-      </c>
       <c r="Q82" t="b">
+        <v>1</v>
+      </c>
+      <c r="R82" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5970,33 +6218,36 @@
         <v>3</v>
       </c>
       <c r="J83" t="n">
+        <v>0</v>
+      </c>
+      <c r="K83" t="n">
         <v>2</v>
       </c>
-      <c r="K83" t="n">
+      <c r="L83" t="n">
         <v>304.8</v>
       </c>
-      <c r="L83" t="n">
+      <c r="M83" t="n">
         <v>277</v>
       </c>
-      <c r="M83" t="inlineStr">
+      <c r="N83" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N83" t="inlineStr">
+      <c r="O83" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O83" t="inlineStr">
+      <c r="P83" t="inlineStr">
         <is>
           <t>Eatx</t>
         </is>
       </c>
-      <c r="P83" t="b">
-        <v>1</v>
-      </c>
       <c r="Q83" t="b">
+        <v>1</v>
+      </c>
+      <c r="R83" t="b">
         <v>1</v>
       </c>
     </row>
@@ -6037,33 +6288,36 @@
         <v>6</v>
       </c>
       <c r="J84" t="n">
+        <v>0</v>
+      </c>
+      <c r="K84" t="n">
         <v>2</v>
-      </c>
-      <c r="K84" t="n">
-        <v>243.84</v>
       </c>
       <c r="L84" t="n">
         <v>243.84</v>
       </c>
-      <c r="M84" t="inlineStr">
+      <c r="M84" t="n">
+        <v>243.84</v>
+      </c>
+      <c r="N84" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N84" t="inlineStr">
+      <c r="O84" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O84" t="inlineStr">
+      <c r="P84" t="inlineStr">
         <is>
           <t>Matx</t>
         </is>
       </c>
-      <c r="P84" t="b">
-        <v>1</v>
-      </c>
       <c r="Q84" t="b">
+        <v>1</v>
+      </c>
+      <c r="R84" t="b">
         <v>1</v>
       </c>
     </row>
@@ -6104,33 +6358,36 @@
         <v>8</v>
       </c>
       <c r="J85" t="n">
+        <v>0</v>
+      </c>
+      <c r="K85" t="n">
         <v>2</v>
       </c>
-      <c r="K85" t="n">
+      <c r="L85" t="n">
         <v>304.8</v>
       </c>
-      <c r="L85" t="n">
+      <c r="M85" t="n">
         <v>243.84</v>
       </c>
-      <c r="M85" t="inlineStr">
+      <c r="N85" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N85" t="inlineStr">
+      <c r="O85" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O85" t="inlineStr">
+      <c r="P85" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P85" t="b">
-        <v>1</v>
-      </c>
       <c r="Q85" t="b">
+        <v>1</v>
+      </c>
+      <c r="R85" t="b">
         <v>1</v>
       </c>
     </row>
@@ -6171,33 +6428,36 @@
         <v>8</v>
       </c>
       <c r="J86" t="n">
+        <v>0</v>
+      </c>
+      <c r="K86" t="n">
         <v>2</v>
       </c>
-      <c r="K86" t="n">
+      <c r="L86" t="n">
         <v>304.8</v>
       </c>
-      <c r="L86" t="n">
+      <c r="M86" t="n">
         <v>243.84</v>
       </c>
-      <c r="M86" t="inlineStr">
+      <c r="N86" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N86" t="inlineStr">
+      <c r="O86" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O86" t="inlineStr">
+      <c r="P86" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P86" t="b">
-        <v>1</v>
-      </c>
       <c r="Q86" t="b">
+        <v>1</v>
+      </c>
+      <c r="R86" t="b">
         <v>1</v>
       </c>
     </row>
@@ -6238,33 +6498,36 @@
         <v>8</v>
       </c>
       <c r="J87" t="n">
+        <v>0</v>
+      </c>
+      <c r="K87" t="n">
         <v>2</v>
       </c>
-      <c r="K87" t="n">
+      <c r="L87" t="n">
         <v>304.8</v>
       </c>
-      <c r="L87" t="n">
+      <c r="M87" t="n">
         <v>243.84</v>
       </c>
-      <c r="M87" t="inlineStr">
+      <c r="N87" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N87" t="inlineStr">
+      <c r="O87" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O87" t="inlineStr">
+      <c r="P87" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P87" t="b">
-        <v>1</v>
-      </c>
       <c r="Q87" t="b">
+        <v>1</v>
+      </c>
+      <c r="R87" t="b">
         <v>1</v>
       </c>
     </row>
@@ -6305,33 +6568,36 @@
         <v>8</v>
       </c>
       <c r="J88" t="n">
+        <v>0</v>
+      </c>
+      <c r="K88" t="n">
         <v>2</v>
       </c>
-      <c r="K88" t="n">
+      <c r="L88" t="n">
         <v>304.8</v>
       </c>
-      <c r="L88" t="n">
+      <c r="M88" t="n">
         <v>243.84</v>
       </c>
-      <c r="M88" t="inlineStr">
+      <c r="N88" t="inlineStr">
         <is>
           <t>Ddr5</t>
         </is>
       </c>
-      <c r="N88" t="inlineStr">
+      <c r="O88" t="inlineStr">
         <is>
           <t>UDimm</t>
         </is>
       </c>
-      <c r="O88" t="inlineStr">
+      <c r="P88" t="inlineStr">
         <is>
           <t>Atx</t>
         </is>
       </c>
-      <c r="P88" t="b">
-        <v>1</v>
-      </c>
       <c r="Q88" t="b">
+        <v>1</v>
+      </c>
+      <c r="R88" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>